<commit_message>
Refactor packet handling and table updates in GUI
Updated packet parsing in j2050_gui.py to use 'PACKET:' prefix instead of 'Decoded:'. Adjusted table column indices for RSSI, SNR, and frequency shift, and changed timestamp handling to use formatted datetime strings. Fixed extraction of task_ID in GS_task.py and corrected timestamp usage in Jdata.py for packet saving. Updated database and export files to reflect these changes.
</commit_message>
<xml_diff>
--- a/packets_export.xlsx
+++ b/packets_export.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M6"/>
+  <dimension ref="A1:M12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -500,23 +500,23 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2025-10-11 18:07:59</t>
+          <t>2025-10-15 13:07:33</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>b'\x01\xaa3\x0cgt\x85\xda\xd2\xea\x8b\x07\xc2\xdf\x00\x00\xc1(\x00\x00C\x8d\x08\x92\x00\x00\x00\x00'</t>
+          <t>b'\x01U3\x0cgt\x86i|e\xcc\xdb\xc2X\x00\x00A$\x00\x00\xc4\xe7\x9a\xae'</t>
         </is>
       </c>
       <c r="D2" t="n">
         <v>1</v>
       </c>
       <c r="E2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F2" t="n">
         <v>51</v>
@@ -525,47 +525,47 @@
         <v>12</v>
       </c>
       <c r="H2" t="n">
-        <v>1735689690</v>
+        <v>1735689833</v>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>3538586375</t>
+          <t>2087046363</t>
         </is>
       </c>
       <c r="J2" t="n">
-        <v>-70</v>
+        <v>-50</v>
       </c>
       <c r="K2" t="n">
-        <v>10.1</v>
+        <v>10.75</v>
       </c>
       <c r="L2" t="n">
-        <v>0</v>
+        <v>1848.64</v>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>Dati telemetria</t>
+          <t>test</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2025-10-11 18:08:47</t>
+          <t>2025-10-15 13:21:55</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>b'\x01\xaa3\x0cgt\x85\xda\xd2\xea\x8b\x07\xc2\xdf\x00\x00\xc1(\x00\x00C\x8d\x08\x92\x00\x00\x00\x00'</t>
+          <t>b'\x01U3\x0cgt\x89\xc7\x11\xdb\xb7\xb1\xc2X\x00\x00A$\x00\x00\xc4\x97 C'</t>
         </is>
       </c>
       <c r="D3" t="n">
         <v>1</v>
       </c>
       <c r="E3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F3" t="n">
         <v>51</v>
@@ -574,172 +574,460 @@
         <v>12</v>
       </c>
       <c r="H3" t="n">
-        <v>1735689690</v>
+        <v>1735690695</v>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>3538586375</t>
+          <t>299612081</t>
         </is>
       </c>
       <c r="J3" t="n">
-        <v>-70</v>
+        <v>-50</v>
       </c>
       <c r="K3" t="n">
-        <v>10.1</v>
+        <v>10.5</v>
       </c>
       <c r="L3" t="n">
-        <v>0</v>
+        <v>1202.72</v>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>Dati telemetria</t>
+          <t>test3</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2025-10-11 18:12:09</t>
+          <t>2025-10-15 13:23:36</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>b'\x01\xaa3\x0cgt\x85\xda\xd2\xea\x8b\x07\xc2\xdf\x00\x00\xc1(\x00\x00C\x8d\x08\x92\x00\x00\x00\x00'</t>
+          <t>b'\x01U1\x01gt\x8a,\x03\xfbz_\x18'</t>
         </is>
       </c>
       <c r="D4" t="n">
         <v>1</v>
       </c>
       <c r="E4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F4" t="n">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="G4" t="n">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="H4" t="n">
-        <v>1735689690</v>
+        <v>1735690796</v>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>3538586375</t>
+          <t>66812511</t>
         </is>
       </c>
       <c r="J4" t="n">
-        <v>-70</v>
+        <v>-54</v>
       </c>
       <c r="K4" t="n">
-        <v>10.1</v>
+        <v>9.75</v>
       </c>
       <c r="L4" t="n">
-        <v>0</v>
+        <v>1274.02</v>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>Dati telemetria</t>
+          <t>test4</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2025-10-11 18:18:08</t>
+          <t>2025-10-15 13:23:41</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>b'\x01\xaa3\x0cgt\x85\xda\xd2\xea\x8b\x07\xc2\xdf\x00\x00\xc1(\x00\x00C\x8d\x08\x92\x00\x00\x00\x00'</t>
+          <t>b'\x01U1\x01gt\x8a1\x9a\x02\xf4\xa5\x18'</t>
         </is>
       </c>
       <c r="D5" t="n">
         <v>1</v>
       </c>
       <c r="E5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F5" t="n">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="G5" t="n">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="H5" t="n">
-        <v>1735689690</v>
+        <v>1735690801</v>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>3538586375</t>
+          <t>2583884965</t>
         </is>
       </c>
       <c r="J5" t="n">
-        <v>-70</v>
+        <v>-54</v>
       </c>
       <c r="K5" t="n">
-        <v>10.1</v>
+        <v>10</v>
       </c>
       <c r="L5" t="n">
-        <v>0</v>
+        <v>1204.81</v>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>Dati telemetria</t>
+          <t>test4</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2025-10-11 18:20:40</t>
+          <t>2025-10-15 13:26:21</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>b'\x01\xaa3\x0cgt\x85\xda\xd2\xea\x8b\x07\xc2\xdf\x00\x00\xc1(\x00\x00C\x8d\x08\x92\x00\x00\x00\x00'</t>
+          <t>b'\x01U1\x01gt\x8a\xd1;K\xfd\x8c\x18'</t>
         </is>
       </c>
       <c r="D6" t="n">
         <v>1</v>
       </c>
       <c r="E6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F6" t="n">
+        <v>49</v>
+      </c>
+      <c r="G6" t="n">
+        <v>1</v>
+      </c>
+      <c r="H6" t="n">
+        <v>1735690961</v>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>994835852</t>
+        </is>
+      </c>
+      <c r="J6" t="n">
+        <v>-53</v>
+      </c>
+      <c r="K6" t="n">
+        <v>10.5</v>
+      </c>
+      <c r="L6" t="n">
+        <v>298.84</v>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>test5</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>11</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>2025-10-15 13:26:26</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>b'\x01U1\x01gt\x8a\xd6/ew\x87\x18'</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>1</v>
+      </c>
+      <c r="E7" t="n">
+        <v>0</v>
+      </c>
+      <c r="F7" t="n">
+        <v>49</v>
+      </c>
+      <c r="G7" t="n">
+        <v>1</v>
+      </c>
+      <c r="H7" t="n">
+        <v>1735690966</v>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>795178887</t>
+        </is>
+      </c>
+      <c r="J7" t="n">
+        <v>-54</v>
+      </c>
+      <c r="K7" t="n">
+        <v>10.5</v>
+      </c>
+      <c r="L7" t="n">
+        <v>246.42</v>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>test5</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>12</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>2025-10-15 13:28:54</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>b'\x01U1\x01gt\x8bk\x96\xe2\x03u\x18'</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F8" t="n">
+        <v>49</v>
+      </c>
+      <c r="G8" t="n">
+        <v>1</v>
+      </c>
+      <c r="H8" t="n">
+        <v>1735691115</v>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>2531394421</t>
+        </is>
+      </c>
+      <c r="J8" t="n">
+        <v>-54</v>
+      </c>
+      <c r="K8" t="n">
+        <v>10.25</v>
+      </c>
+      <c r="L8" t="n">
+        <v>714.08</v>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>test8</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>13</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>2025-10-15 13:28:59</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>b'\x01U1\x01gt\x8bpO\xc4\xae\xeb\x18'</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>1</v>
+      </c>
+      <c r="E9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F9" t="n">
+        <v>49</v>
+      </c>
+      <c r="G9" t="n">
+        <v>1</v>
+      </c>
+      <c r="H9" t="n">
+        <v>1735691120</v>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>1338289899</t>
+        </is>
+      </c>
+      <c r="J9" t="n">
+        <v>-53</v>
+      </c>
+      <c r="K9" t="n">
+        <v>10.25</v>
+      </c>
+      <c r="L9" t="n">
+        <v>691.01</v>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>test8</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>14</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>2025-10-15 15:49:01</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>b'\x01U3\x0cgt\x90!\xed\xfc\xa7s\xc2\\\x00\x00A,\x00\x00\xc4\xf4/\xe8'</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>1</v>
+      </c>
+      <c r="E10" t="n">
+        <v>0</v>
+      </c>
+      <c r="F10" t="n">
         <v>51</v>
       </c>
-      <c r="G6" t="n">
+      <c r="G10" t="n">
         <v>12</v>
       </c>
-      <c r="H6" t="n">
-        <v>1735689690</v>
-      </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>3538586375</t>
-        </is>
-      </c>
-      <c r="J6" t="n">
-        <v>-70</v>
-      </c>
-      <c r="K6" t="n">
-        <v>10.1</v>
-      </c>
-      <c r="L6" t="n">
+      <c r="H10" t="n">
+        <v>1735692321</v>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>3992758131</t>
+        </is>
+      </c>
+      <c r="J10" t="n">
+        <v>-49</v>
+      </c>
+      <c r="K10" t="n">
+        <v>10.5</v>
+      </c>
+      <c r="L10" t="n">
+        <v>1945.11</v>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>qwe</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>15</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>2025-10-15 15:50:42</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>b'\x10U\x1a\x00h\xef\xa6\xad\xfaX\x9cQ'</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>16</v>
+      </c>
+      <c r="E11" t="n">
         <v>0</v>
       </c>
-      <c r="M6" t="inlineStr">
-        <is>
-          <t>Dati telemetria</t>
+      <c r="F11" t="n">
+        <v>26</v>
+      </c>
+      <c r="G11" t="n">
+        <v>0</v>
+      </c>
+      <c r="H11" t="n">
+        <v>1760536237</v>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>4200111185</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr"/>
+      <c r="K11" t="inlineStr"/>
+      <c r="L11" t="inlineStr"/>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>a</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>16</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>2025-10-15 15:50:43</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>b'\x01U3\x0cgt\x90\x87\xc8\n\xe7\xd2\xc2\\\x00\x00A,\x00\x00\xc4\xf2\x9dA'</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>1</v>
+      </c>
+      <c r="E12" t="n">
+        <v>0</v>
+      </c>
+      <c r="F12" t="n">
+        <v>51</v>
+      </c>
+      <c r="G12" t="n">
+        <v>12</v>
+      </c>
+      <c r="H12" t="n">
+        <v>1735692423</v>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>3356157906</t>
+        </is>
+      </c>
+      <c r="J12" t="n">
+        <v>-50</v>
+      </c>
+      <c r="K12" t="n">
+        <v>10.25</v>
+      </c>
+      <c r="L12" t="n">
+        <v>1934.62</v>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>a</t>
         </is>
       </c>
     </row>
@@ -754,7 +1042,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D6"/>
+  <dimension ref="A1:D10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -847,6 +1135,62 @@
       </c>
       <c r="D6" t="n">
         <v>282.0669555664062</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" t="n">
+        <v>-54</v>
+      </c>
+      <c r="C7" t="n">
+        <v>10.25</v>
+      </c>
+      <c r="D7" t="n">
+        <v>-1852.833740234375</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" t="n">
+        <v>-54</v>
+      </c>
+      <c r="C8" t="n">
+        <v>10.25</v>
+      </c>
+      <c r="D8" t="n">
+        <v>-1209.008178710938</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>14</v>
+      </c>
+      <c r="B9" t="n">
+        <v>-55</v>
+      </c>
+      <c r="C9" t="n">
+        <v>10.75</v>
+      </c>
+      <c r="D9" t="n">
+        <v>-1953.4970703125</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>16</v>
+      </c>
+      <c r="B10" t="n">
+        <v>-55</v>
+      </c>
+      <c r="C10" t="n">
+        <v>10.75</v>
+      </c>
+      <c r="D10" t="n">
+        <v>-1940.914184570312</v>
       </c>
     </row>
   </sheetData>
@@ -891,7 +1235,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B1"/>
+  <dimension ref="A1:B7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -906,6 +1250,58 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>8</v>
+      </c>
+      <c r="B2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>9</v>
+      </c>
+      <c r="B3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>10</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>b'\x00\x00\x00\x00\x00\x00\x00\x00\x00\x00\x00\x00\x00\x00\x00\x00\x00\x00\x00\x00\x00\x00\x00\x00'</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>11</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>b'\x00\x00\x00\x00\x00\x00\x00\x00\x00\x00\x00\x00\x00\x00\x00\x00\x00\x00\x00\x00\x00\x00\x00\x00'</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>12</v>
+      </c>
+      <c r="B6" t="n">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>13</v>
+      </c>
+      <c r="B7" t="n">
+        <v>24</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Use UTC timestamps for TEC and TER events
Replaced local time with UTC for logging sent TEC and received TER events in the GUI. This ensures consistent timestamping across different time zones.
</commit_message>
<xml_diff>
--- a/packets_export.xlsx
+++ b/packets_export.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M91"/>
+  <dimension ref="A1:M94"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5085,6 +5085,159 @@
       <c r="M91" t="inlineStr">
         <is>
           <t>histo2</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="n">
+        <v>91</v>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>2025-10-16 09:08:55</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>b'\x01U3\x0cgt\x86\xdd\x9f\xa8\xa6\xe9\xc2\x84\x00\x00A\x14\x00\x00DYQ@'</t>
+        </is>
+      </c>
+      <c r="D92" t="n">
+        <v>1</v>
+      </c>
+      <c r="E92" t="n">
+        <v>0</v>
+      </c>
+      <c r="F92" t="n">
+        <v>51</v>
+      </c>
+      <c r="G92" t="n">
+        <v>12</v>
+      </c>
+      <c r="H92" t="inlineStr">
+        <is>
+          <t>2025-01-01 00:05:49</t>
+        </is>
+      </c>
+      <c r="I92" t="inlineStr">
+        <is>
+          <t>2678630121</t>
+        </is>
+      </c>
+      <c r="J92" t="n">
+        <v>-63</v>
+      </c>
+      <c r="K92" t="n">
+        <v>12.75</v>
+      </c>
+      <c r="L92" t="n">
+        <v>-869.27</v>
+      </c>
+      <c r="M92" t="inlineStr">
+        <is>
+          <t>test_UTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="n">
+        <v>92</v>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>2025-10-16 09:13:03</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>b'\x01U3\x0ch\xf0\xb6Z\xce\xf0\x0f\xf6\xc2\x90\x00\x00A\x14\x00\x00D\x9aE\x91'</t>
+        </is>
+      </c>
+      <c r="D93" t="n">
+        <v>1</v>
+      </c>
+      <c r="E93" t="n">
+        <v>0</v>
+      </c>
+      <c r="F93" t="n">
+        <v>51</v>
+      </c>
+      <c r="G93" t="n">
+        <v>12</v>
+      </c>
+      <c r="H93" t="inlineStr">
+        <is>
+          <t>2025-10-16 09:09:46</t>
+        </is>
+      </c>
+      <c r="I93" t="inlineStr">
+        <is>
+          <t>3471839222</t>
+        </is>
+      </c>
+      <c r="J93" t="n">
+        <v>-62</v>
+      </c>
+      <c r="K93" t="n">
+        <v>10</v>
+      </c>
+      <c r="L93" t="n">
+        <v>-1236.27</v>
+      </c>
+      <c r="M93" t="inlineStr">
+        <is>
+          <t>k</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="n">
+        <v>93</v>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>2025-10-16 09:13:29</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>b'\x01U3\x0ch\xf0\xb6s\xc1-\xff\xcd\xc2\x94\x00\x00A4\x00\x00D\x9aE\x91'</t>
+        </is>
+      </c>
+      <c r="D94" t="n">
+        <v>1</v>
+      </c>
+      <c r="E94" t="n">
+        <v>0</v>
+      </c>
+      <c r="F94" t="n">
+        <v>51</v>
+      </c>
+      <c r="G94" t="n">
+        <v>12</v>
+      </c>
+      <c r="H94" t="inlineStr">
+        <is>
+          <t>2025-10-16 09:10:11</t>
+        </is>
+      </c>
+      <c r="I94" t="inlineStr">
+        <is>
+          <t>3241017293</t>
+        </is>
+      </c>
+      <c r="J94" t="n">
+        <v>-76</v>
+      </c>
+      <c r="K94" t="n">
+        <v>11.25</v>
+      </c>
+      <c r="L94" t="n">
+        <v>-1238.37</v>
+      </c>
+      <c r="M94" t="inlineStr">
+        <is>
+          <t>kk</t>
         </is>
       </c>
     </row>
@@ -5099,7 +5252,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D91"/>
+  <dimension ref="A1:D94"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6382,6 +6535,48 @@
       </c>
       <c r="D91" t="n">
         <v>1383.07177734375</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="n">
+        <v>91</v>
+      </c>
+      <c r="B92" t="n">
+        <v>-66</v>
+      </c>
+      <c r="C92" t="n">
+        <v>9.25</v>
+      </c>
+      <c r="D92" t="n">
+        <v>869.26953125</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="n">
+        <v>92</v>
+      </c>
+      <c r="B93" t="n">
+        <v>-72</v>
+      </c>
+      <c r="C93" t="n">
+        <v>9.25</v>
+      </c>
+      <c r="D93" t="n">
+        <v>1234.173950195312</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="n">
+        <v>93</v>
+      </c>
+      <c r="B94" t="n">
+        <v>-74</v>
+      </c>
+      <c r="C94" t="n">
+        <v>11.25</v>
+      </c>
+      <c r="D94" t="n">
+        <v>1234.173950195312</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Redesign Jdata.py GUI with advanced filtering and details
Refactored the packet database viewer to use a modern grid-based layout with advanced filtering options (by type, GS ID, date, and comment), improved packet detail display, and multi-selection deletion. Added helper functions in GS_task.py for label/ID lookups, and updated the database and export files accordingly.
</commit_message>
<xml_diff>
--- a/packets_export.xlsx
+++ b/packets_export.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M94"/>
+  <dimension ref="A1:M84"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4728,516 +4728,6 @@
       <c r="M84" t="inlineStr">
         <is>
           <t>histo2</t>
-        </is>
-      </c>
-    </row>
-    <row r="85">
-      <c r="A85" t="n">
-        <v>84</v>
-      </c>
-      <c r="B85" t="inlineStr">
-        <is>
-          <t>2025-10-15 22:26:03</t>
-        </is>
-      </c>
-      <c r="C85" t="inlineStr">
-        <is>
-          <t>b'\x01U3\x0ch\xf0\x03#\\\x12\x907\xc2\x94\x00\x00A(\x00\x00D\xadh\x83'</t>
-        </is>
-      </c>
-      <c r="D85" t="n">
-        <v>1</v>
-      </c>
-      <c r="E85" t="n">
-        <v>0</v>
-      </c>
-      <c r="F85" t="n">
-        <v>51</v>
-      </c>
-      <c r="G85" t="n">
-        <v>12</v>
-      </c>
-      <c r="H85" t="inlineStr">
-        <is>
-          <t>2025-10-15 20:25:07</t>
-        </is>
-      </c>
-      <c r="I85" t="inlineStr">
-        <is>
-          <t>1544720439</t>
-        </is>
-      </c>
-      <c r="J85" t="n">
-        <v>-65</v>
-      </c>
-      <c r="K85" t="n">
-        <v>13</v>
-      </c>
-      <c r="L85" t="n">
-        <v>-1389.36</v>
-      </c>
-      <c r="M85" t="inlineStr">
-        <is>
-          <t>histo2</t>
-        </is>
-      </c>
-    </row>
-    <row r="86">
-      <c r="A86" t="n">
-        <v>85</v>
-      </c>
-      <c r="B86" t="inlineStr">
-        <is>
-          <t>2025-10-15 22:26:05</t>
-        </is>
-      </c>
-      <c r="C86" t="inlineStr">
-        <is>
-          <t>b'\x01U3\x0ch\xf0\x03%]\xfa\x19\x94\xc2\x96\x00\x00A8\x00\x00D\xad%h'</t>
-        </is>
-      </c>
-      <c r="D86" t="n">
-        <v>1</v>
-      </c>
-      <c r="E86" t="n">
-        <v>0</v>
-      </c>
-      <c r="F86" t="n">
-        <v>51</v>
-      </c>
-      <c r="G86" t="n">
-        <v>12</v>
-      </c>
-      <c r="H86" t="inlineStr">
-        <is>
-          <t>2025-10-15 20:25:09</t>
-        </is>
-      </c>
-      <c r="I86" t="inlineStr">
-        <is>
-          <t>1576671636</t>
-        </is>
-      </c>
-      <c r="J86" t="n">
-        <v>-64</v>
-      </c>
-      <c r="K86" t="n">
-        <v>12.75</v>
-      </c>
-      <c r="L86" t="n">
-        <v>-1389.36</v>
-      </c>
-      <c r="M86" t="inlineStr">
-        <is>
-          <t>histo2</t>
-        </is>
-      </c>
-    </row>
-    <row r="87">
-      <c r="A87" t="n">
-        <v>86</v>
-      </c>
-      <c r="B87" t="inlineStr">
-        <is>
-          <t>2025-10-15 22:26:08</t>
-        </is>
-      </c>
-      <c r="C87" t="inlineStr">
-        <is>
-          <t>b"\x01U3\x0ch\xf0\x03'\xcb\n'\xde\xc2\x98\x00\x00A(\x00\x00D\xadh\x83"</t>
-        </is>
-      </c>
-      <c r="D87" t="n">
-        <v>1</v>
-      </c>
-      <c r="E87" t="n">
-        <v>0</v>
-      </c>
-      <c r="F87" t="n">
-        <v>51</v>
-      </c>
-      <c r="G87" t="n">
-        <v>12</v>
-      </c>
-      <c r="H87" t="inlineStr">
-        <is>
-          <t>2025-10-15 20:25:11</t>
-        </is>
-      </c>
-      <c r="I87" t="inlineStr">
-        <is>
-          <t>3406440414</t>
-        </is>
-      </c>
-      <c r="J87" t="n">
-        <v>-66</v>
-      </c>
-      <c r="K87" t="n">
-        <v>12.5</v>
-      </c>
-      <c r="L87" t="n">
-        <v>-1391.46</v>
-      </c>
-      <c r="M87" t="inlineStr">
-        <is>
-          <t>histo2</t>
-        </is>
-      </c>
-    </row>
-    <row r="88">
-      <c r="A88" t="n">
-        <v>87</v>
-      </c>
-      <c r="B88" t="inlineStr">
-        <is>
-          <t>2025-10-15 22:26:10</t>
-        </is>
-      </c>
-      <c r="C88" t="inlineStr">
-        <is>
-          <t>b'\x01U3\x0ch\xf0\x03)\x03\x8c\xdd=\xc2\x96\x00\x00A8\x00\x00D\xac\xe2L'</t>
-        </is>
-      </c>
-      <c r="D88" t="n">
-        <v>1</v>
-      </c>
-      <c r="E88" t="n">
-        <v>0</v>
-      </c>
-      <c r="F88" t="n">
-        <v>51</v>
-      </c>
-      <c r="G88" t="n">
-        <v>12</v>
-      </c>
-      <c r="H88" t="inlineStr">
-        <is>
-          <t>2025-10-15 20:25:13</t>
-        </is>
-      </c>
-      <c r="I88" t="inlineStr">
-        <is>
-          <t>59563325</t>
-        </is>
-      </c>
-      <c r="J88" t="n">
-        <v>-65</v>
-      </c>
-      <c r="K88" t="n">
-        <v>12.75</v>
-      </c>
-      <c r="L88" t="n">
-        <v>-1387.27</v>
-      </c>
-      <c r="M88" t="inlineStr">
-        <is>
-          <t>histo2</t>
-        </is>
-      </c>
-    </row>
-    <row r="89">
-      <c r="A89" t="n">
-        <v>88</v>
-      </c>
-      <c r="B89" t="inlineStr">
-        <is>
-          <t>2025-10-15 22:26:12</t>
-        </is>
-      </c>
-      <c r="C89" t="inlineStr">
-        <is>
-          <t>b'\x01U3\x0ch\xf0\x03+\xf8t\x96O\xc2\x98\x00\x00A(\x00\x00D\xad%h'</t>
-        </is>
-      </c>
-      <c r="D89" t="n">
-        <v>1</v>
-      </c>
-      <c r="E89" t="n">
-        <v>0</v>
-      </c>
-      <c r="F89" t="n">
-        <v>51</v>
-      </c>
-      <c r="G89" t="n">
-        <v>12</v>
-      </c>
-      <c r="H89" t="inlineStr">
-        <is>
-          <t>2025-10-15 20:25:15</t>
-        </is>
-      </c>
-      <c r="I89" t="inlineStr">
-        <is>
-          <t>4168390223</t>
-        </is>
-      </c>
-      <c r="J89" t="n">
-        <v>-65</v>
-      </c>
-      <c r="K89" t="n">
-        <v>12.75</v>
-      </c>
-      <c r="L89" t="n">
-        <v>-1389.36</v>
-      </c>
-      <c r="M89" t="inlineStr">
-        <is>
-          <t>histo2</t>
-        </is>
-      </c>
-    </row>
-    <row r="90">
-      <c r="A90" t="n">
-        <v>89</v>
-      </c>
-      <c r="B90" t="inlineStr">
-        <is>
-          <t>2025-10-15 22:26:14</t>
-        </is>
-      </c>
-      <c r="C90" t="inlineStr">
-        <is>
-          <t>b'\x01U3\x0ch\xf0\x03-\xba~(\x10\xc2\x94\x00\x00A4\x00\x00D\xac\xe2L'</t>
-        </is>
-      </c>
-      <c r="D90" t="n">
-        <v>1</v>
-      </c>
-      <c r="E90" t="n">
-        <v>0</v>
-      </c>
-      <c r="F90" t="n">
-        <v>51</v>
-      </c>
-      <c r="G90" t="n">
-        <v>12</v>
-      </c>
-      <c r="H90" t="inlineStr">
-        <is>
-          <t>2025-10-15 20:25:17</t>
-        </is>
-      </c>
-      <c r="I90" t="inlineStr">
-        <is>
-          <t>3128829968</t>
-        </is>
-      </c>
-      <c r="J90" t="n">
-        <v>-66</v>
-      </c>
-      <c r="K90" t="n">
-        <v>13</v>
-      </c>
-      <c r="L90" t="n">
-        <v>-1387.27</v>
-      </c>
-      <c r="M90" t="inlineStr">
-        <is>
-          <t>histo2</t>
-        </is>
-      </c>
-    </row>
-    <row r="91">
-      <c r="A91" t="n">
-        <v>90</v>
-      </c>
-      <c r="B91" t="inlineStr">
-        <is>
-          <t>2025-10-15 22:26:16</t>
-        </is>
-      </c>
-      <c r="C91" t="inlineStr">
-        <is>
-          <t>b'\x01U3\x0ch\xf0\x03/8\x14\xc1\xce\xc2\x96\x00\x00A0\x00\x00D\xac\xe2L'</t>
-        </is>
-      </c>
-      <c r="D91" t="n">
-        <v>1</v>
-      </c>
-      <c r="E91" t="n">
-        <v>0</v>
-      </c>
-      <c r="F91" t="n">
-        <v>51</v>
-      </c>
-      <c r="G91" t="n">
-        <v>12</v>
-      </c>
-      <c r="H91" t="inlineStr">
-        <is>
-          <t>2025-10-15 20:25:19</t>
-        </is>
-      </c>
-      <c r="I91" t="inlineStr">
-        <is>
-          <t>940884430</t>
-        </is>
-      </c>
-      <c r="J91" t="n">
-        <v>-66</v>
-      </c>
-      <c r="K91" t="n">
-        <v>13</v>
-      </c>
-      <c r="L91" t="n">
-        <v>-1387.27</v>
-      </c>
-      <c r="M91" t="inlineStr">
-        <is>
-          <t>histo2</t>
-        </is>
-      </c>
-    </row>
-    <row r="92">
-      <c r="A92" t="n">
-        <v>91</v>
-      </c>
-      <c r="B92" t="inlineStr">
-        <is>
-          <t>2025-10-16 09:08:55</t>
-        </is>
-      </c>
-      <c r="C92" t="inlineStr">
-        <is>
-          <t>b'\x01U3\x0cgt\x86\xdd\x9f\xa8\xa6\xe9\xc2\x84\x00\x00A\x14\x00\x00DYQ@'</t>
-        </is>
-      </c>
-      <c r="D92" t="n">
-        <v>1</v>
-      </c>
-      <c r="E92" t="n">
-        <v>0</v>
-      </c>
-      <c r="F92" t="n">
-        <v>51</v>
-      </c>
-      <c r="G92" t="n">
-        <v>12</v>
-      </c>
-      <c r="H92" t="inlineStr">
-        <is>
-          <t>2025-01-01 00:05:49</t>
-        </is>
-      </c>
-      <c r="I92" t="inlineStr">
-        <is>
-          <t>2678630121</t>
-        </is>
-      </c>
-      <c r="J92" t="n">
-        <v>-63</v>
-      </c>
-      <c r="K92" t="n">
-        <v>12.75</v>
-      </c>
-      <c r="L92" t="n">
-        <v>-869.27</v>
-      </c>
-      <c r="M92" t="inlineStr">
-        <is>
-          <t>test_UTC</t>
-        </is>
-      </c>
-    </row>
-    <row r="93">
-      <c r="A93" t="n">
-        <v>92</v>
-      </c>
-      <c r="B93" t="inlineStr">
-        <is>
-          <t>2025-10-16 09:13:03</t>
-        </is>
-      </c>
-      <c r="C93" t="inlineStr">
-        <is>
-          <t>b'\x01U3\x0ch\xf0\xb6Z\xce\xf0\x0f\xf6\xc2\x90\x00\x00A\x14\x00\x00D\x9aE\x91'</t>
-        </is>
-      </c>
-      <c r="D93" t="n">
-        <v>1</v>
-      </c>
-      <c r="E93" t="n">
-        <v>0</v>
-      </c>
-      <c r="F93" t="n">
-        <v>51</v>
-      </c>
-      <c r="G93" t="n">
-        <v>12</v>
-      </c>
-      <c r="H93" t="inlineStr">
-        <is>
-          <t>2025-10-16 09:09:46</t>
-        </is>
-      </c>
-      <c r="I93" t="inlineStr">
-        <is>
-          <t>3471839222</t>
-        </is>
-      </c>
-      <c r="J93" t="n">
-        <v>-62</v>
-      </c>
-      <c r="K93" t="n">
-        <v>10</v>
-      </c>
-      <c r="L93" t="n">
-        <v>-1236.27</v>
-      </c>
-      <c r="M93" t="inlineStr">
-        <is>
-          <t>k</t>
-        </is>
-      </c>
-    </row>
-    <row r="94">
-      <c r="A94" t="n">
-        <v>93</v>
-      </c>
-      <c r="B94" t="inlineStr">
-        <is>
-          <t>2025-10-16 09:13:29</t>
-        </is>
-      </c>
-      <c r="C94" t="inlineStr">
-        <is>
-          <t>b'\x01U3\x0ch\xf0\xb6s\xc1-\xff\xcd\xc2\x94\x00\x00A4\x00\x00D\x9aE\x91'</t>
-        </is>
-      </c>
-      <c r="D94" t="n">
-        <v>1</v>
-      </c>
-      <c r="E94" t="n">
-        <v>0</v>
-      </c>
-      <c r="F94" t="n">
-        <v>51</v>
-      </c>
-      <c r="G94" t="n">
-        <v>12</v>
-      </c>
-      <c r="H94" t="inlineStr">
-        <is>
-          <t>2025-10-16 09:10:11</t>
-        </is>
-      </c>
-      <c r="I94" t="inlineStr">
-        <is>
-          <t>3241017293</t>
-        </is>
-      </c>
-      <c r="J94" t="n">
-        <v>-76</v>
-      </c>
-      <c r="K94" t="n">
-        <v>11.25</v>
-      </c>
-      <c r="L94" t="n">
-        <v>-1238.37</v>
-      </c>
-      <c r="M94" t="inlineStr">
-        <is>
-          <t>kk</t>
         </is>
       </c>
     </row>
@@ -5252,7 +4742,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D94"/>
+  <dimension ref="A1:D89"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6441,142 +5931,72 @@
     </row>
     <row r="85">
       <c r="A85" t="n">
-        <v>84</v>
+        <v>90</v>
       </c>
       <c r="B85" t="n">
-        <v>-74</v>
+        <v>-75</v>
       </c>
       <c r="C85" t="n">
-        <v>10.5</v>
+        <v>11</v>
       </c>
       <c r="D85" t="n">
-        <v>1387.265991210938</v>
+        <v>1383.07177734375</v>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="n">
-        <v>85</v>
+        <v>91</v>
       </c>
       <c r="B86" t="n">
-        <v>-75</v>
+        <v>-66</v>
       </c>
       <c r="C86" t="n">
-        <v>11.5</v>
+        <v>9.25</v>
       </c>
       <c r="D86" t="n">
-        <v>1385.1689453125</v>
+        <v>869.26953125</v>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="n">
-        <v>86</v>
+        <v>92</v>
       </c>
       <c r="B87" t="n">
-        <v>-76</v>
+        <v>-72</v>
       </c>
       <c r="C87" t="n">
-        <v>10.5</v>
+        <v>9.25</v>
       </c>
       <c r="D87" t="n">
-        <v>1387.265991210938</v>
+        <v>1234.173950195312</v>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="n">
-        <v>87</v>
+        <v>93</v>
       </c>
       <c r="B88" t="n">
-        <v>-75</v>
+        <v>-74</v>
       </c>
       <c r="C88" t="n">
-        <v>11.5</v>
+        <v>11.25</v>
       </c>
       <c r="D88" t="n">
-        <v>1383.07177734375</v>
+        <v>1234.173950195312</v>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="n">
-        <v>88</v>
+        <v>94</v>
       </c>
       <c r="B89" t="n">
-        <v>-76</v>
+        <v>-73</v>
       </c>
       <c r="C89" t="n">
-        <v>10.5</v>
+        <v>13.5</v>
       </c>
       <c r="D89" t="n">
-        <v>1385.1689453125</v>
-      </c>
-    </row>
-    <row r="90">
-      <c r="A90" t="n">
-        <v>89</v>
-      </c>
-      <c r="B90" t="n">
-        <v>-74</v>
-      </c>
-      <c r="C90" t="n">
-        <v>11.25</v>
-      </c>
-      <c r="D90" t="n">
-        <v>1383.07177734375</v>
-      </c>
-    </row>
-    <row r="91">
-      <c r="A91" t="n">
-        <v>90</v>
-      </c>
-      <c r="B91" t="n">
-        <v>-75</v>
-      </c>
-      <c r="C91" t="n">
-        <v>11</v>
-      </c>
-      <c r="D91" t="n">
-        <v>1383.07177734375</v>
-      </c>
-    </row>
-    <row r="92">
-      <c r="A92" t="n">
-        <v>91</v>
-      </c>
-      <c r="B92" t="n">
-        <v>-66</v>
-      </c>
-      <c r="C92" t="n">
-        <v>9.25</v>
-      </c>
-      <c r="D92" t="n">
-        <v>869.26953125</v>
-      </c>
-    </row>
-    <row r="93">
-      <c r="A93" t="n">
-        <v>92</v>
-      </c>
-      <c r="B93" t="n">
-        <v>-72</v>
-      </c>
-      <c r="C93" t="n">
-        <v>9.25</v>
-      </c>
-      <c r="D93" t="n">
-        <v>1234.173950195312</v>
-      </c>
-    </row>
-    <row r="94">
-      <c r="A94" t="n">
-        <v>93</v>
-      </c>
-      <c r="B94" t="n">
-        <v>-74</v>
-      </c>
-      <c r="C94" t="n">
-        <v>11.25</v>
-      </c>
-      <c r="D94" t="n">
-        <v>1234.173950195312</v>
+        <v>1167.065063476562</v>
       </c>
     </row>
   </sheetData>

</xml_diff>